<commit_message>
fix contract payment dates and virtual accounts
</commit_message>
<xml_diff>
--- a/db/templates/contracts/contract_client_copy.xlsx
+++ b/db/templates/contracts/contract_client_copy.xlsx
@@ -2419,7 +2419,7 @@
       </c>
       <c r="C33" s="50" t="inlineStr">
         <is>
-          <t>匯款日期</t>
+          <t>預計繳款日</t>
         </is>
       </c>
       <c r="D33" s="51" t="inlineStr">
@@ -2448,7 +2448,7 @@
       </c>
       <c r="C34" s="56" t="inlineStr">
         <is>
-          <t>訂金日期(訂單系統)</t>
+          <t>預計訂金繳款日(訂單系統)</t>
         </is>
       </c>
       <c r="D34" s="57" t="inlineStr">
@@ -2477,12 +2477,12 @@
       </c>
       <c r="C35" s="56" t="inlineStr">
         <is>
-          <t>第一期款入帳日(訂單系統)</t>
+          <t>預計第一期繳款日(訂單系統)</t>
         </is>
       </c>
       <c r="D35" s="213" t="inlineStr">
         <is>
-          <t>服務款項匯款帳號：(代收付)</t>
+          <t>本案專屬虛擬帳號：</t>
         </is>
       </c>
       <c r="E35" s="213" t="n"/>
@@ -2502,12 +2502,12 @@
       </c>
       <c r="C36" s="56" t="inlineStr">
         <is>
-          <t>第二期款入帳日(訂單系統)</t>
+          <t>預計第二期繳款日(訂單系統)</t>
         </is>
       </c>
       <c r="D36" s="62" t="inlineStr">
         <is>
-          <t>還不確定要給哪個帳號</t>
+          <t>案件專屬虛擬帳號(訂單系統)</t>
         </is>
       </c>
       <c r="E36" s="213" t="n"/>
@@ -2527,7 +2527,7 @@
       </c>
       <c r="C37" s="56" t="inlineStr">
         <is>
-          <t>訂金日期(訂單系統)</t>
+          <t>樓層費預計繳款日(訂單系統)</t>
         </is>
       </c>
       <c r="D37" s="213" t="inlineStr">

</xml_diff>

<commit_message>
fix: align issue 327 contract projections
</commit_message>
<xml_diff>
--- a/db/templates/contracts/contract_client_copy.xlsx
+++ b/db/templates/contracts/contract_client_copy.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="客戶契約" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="客戶契約" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'客戶契約'!$A$1:$G$185</definedName>
@@ -28,7 +28,7 @@
     <numFmt numFmtId="170" formatCode="[$-404]General"/>
     <numFmt numFmtId="171" formatCode="[$-404]ggge\年m\月d\日;@"/>
   </numFmts>
-  <fonts count="67">
+  <fonts count="68">
     <font>
       <name val="Noto Sans TC"/>
       <charset val="136"/>
@@ -524,6 +524,12 @@
       <b val="1"/>
       <color rgb="FF000000"/>
       <sz val="11.5"/>
+    </font>
+    <font>
+      <name val="標楷體"/>
+      <b val="1"/>
+      <color theme="1"/>
+      <sz val="14"/>
     </font>
   </fonts>
   <fills count="13">
@@ -600,7 +606,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="13">
+  <borders count="17">
     <border>
       <left/>
       <right/>
@@ -692,6 +698,27 @@
       <bottom style="thin"/>
       <diagonal/>
     </border>
+    <border/>
+    <border>
+      <bottom style="double">
+        <color rgb="00000000"/>
+      </bottom>
+    </border>
+    <border>
+      <right/>
+      <bottom style="double">
+        <color rgb="00000000"/>
+      </bottom>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color rgb="00000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1">
@@ -703,7 +730,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="308">
+  <cellXfs count="316">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -1615,6 +1642,26 @@
     </xf>
     <xf numFmtId="171" fontId="41" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="distributed" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="9" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="168" fontId="17" fillId="2" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="67" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -2012,25 +2059,23 @@
       <c r="F9" s="150" t="n"/>
       <c r="G9" s="150" t="n"/>
     </row>
-    <row r="10" ht="17.15" customHeight="1" s="148">
+    <row r="10" ht="38" customHeight="1" s="148">
       <c r="A10" s="14" t="inlineStr">
         <is>
           <t>服務平台派選服務人員:</t>
         </is>
       </c>
       <c r="B10" s="166" t="n"/>
-      <c r="C10" s="16" t="inlineStr">
+      <c r="C10" s="312" t="inlineStr">
         <is>
           <t>服務人員(綁定好的服務人員)</t>
         </is>
       </c>
-      <c r="E10" s="17" t="inlineStr">
+      <c r="F10" s="313" t="inlineStr">
         <is>
           <t>服務 (以下簡稱受託人乙方)</t>
         </is>
       </c>
-      <c r="F10" s="166" t="n"/>
-      <c r="G10" s="150" t="n"/>
     </row>
     <row r="11" ht="15" customHeight="1" s="148">
       <c r="A11" s="18" t="inlineStr">
@@ -2252,7 +2297,7 @@
       </c>
       <c r="D25" s="150" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t> </t>
         </is>
       </c>
       <c r="E25" s="27" t="inlineStr">
@@ -2435,7 +2480,7 @@
       <c r="F33" s="205" t="n"/>
       <c r="G33" s="205" t="n"/>
     </row>
-    <row r="34" ht="15" customHeight="1" s="148">
+    <row r="34" ht="18" customHeight="1" s="148">
       <c r="A34" s="54" t="inlineStr">
         <is>
           <t>訂金</t>
@@ -2456,13 +2501,11 @@
           <t xml:space="preserve">雇主登記MAIL: </t>
         </is>
       </c>
-      <c r="E34" s="58" t="inlineStr">
+      <c r="E34" s="309" t="inlineStr">
         <is>
           <t>Email(市府表單)</t>
         </is>
       </c>
-      <c r="F34" s="211" t="n"/>
-      <c r="G34" s="211" t="n"/>
     </row>
     <row r="35" ht="15" customHeight="1" s="148">
       <c r="A35" s="54" t="inlineStr">
@@ -2552,7 +2595,7 @@
       </c>
       <c r="C38" s="68" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t> </t>
         </is>
       </c>
       <c r="D38" s="69" t="inlineStr">
@@ -4462,25 +4505,23 @@
       <c r="F180" s="291" t="n"/>
       <c r="G180" s="291" t="n"/>
     </row>
-    <row r="181" ht="15" customHeight="1" s="148">
+    <row r="181" ht="38" customHeight="1" s="148">
       <c r="A181" s="298" t="inlineStr">
         <is>
           <t>服務人員(乙方)：</t>
         </is>
       </c>
-      <c r="B181" s="141">
+      <c r="B181" s="310">
         <f>C10</f>
         <v/>
       </c>
-      <c r="C181" s="304" t="n"/>
-      <c r="D181" s="291" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> (簽章)</t>
-        </is>
-      </c>
-      <c r="E181" s="291" t="n"/>
-      <c r="F181" s="291" t="n"/>
-      <c r="G181" s="291" t="n"/>
+      <c r="C181" s="314" t="n"/>
+      <c r="D181" s="314" t="n"/>
+      <c r="E181" s="315" t="inlineStr">
+        <is>
+          <t>（簽章）</t>
+        </is>
+      </c>
     </row>
     <row r="182" ht="15" customHeight="1" s="148">
       <c r="A182" s="159" t="inlineStr">
@@ -4536,7 +4577,7 @@
       <c r="G185" s="150" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="112">
+  <mergeCells count="116">
     <mergeCell ref="B42:D42"/>
     <mergeCell ref="C80:E80"/>
     <mergeCell ref="E40:G40"/>
@@ -4560,6 +4601,7 @@
     <mergeCell ref="C101:G101"/>
     <mergeCell ref="E28:G28"/>
     <mergeCell ref="A116:G116"/>
+    <mergeCell ref="F10:G10"/>
     <mergeCell ref="C75:E75"/>
     <mergeCell ref="A131:G131"/>
     <mergeCell ref="A156:G156"/>
@@ -4580,14 +4622,18 @@
     <mergeCell ref="A168:G168"/>
     <mergeCell ref="F31:G31"/>
     <mergeCell ref="B3:G3"/>
+    <mergeCell ref="E181:G181"/>
     <mergeCell ref="B95:C95"/>
     <mergeCell ref="C79:E79"/>
     <mergeCell ref="C73:E73"/>
     <mergeCell ref="C63:E63"/>
+    <mergeCell ref="C10:E10"/>
     <mergeCell ref="A32:G32"/>
     <mergeCell ref="C55:E55"/>
     <mergeCell ref="A106:G106"/>
+    <mergeCell ref="B181:D181"/>
     <mergeCell ref="C104:G104"/>
+    <mergeCell ref="E34:G34"/>
     <mergeCell ref="A147:G147"/>
     <mergeCell ref="A161:G161"/>
     <mergeCell ref="A26:F26"/>
@@ -4627,7 +4673,6 @@
     <mergeCell ref="C56:E56"/>
     <mergeCell ref="C88:D88"/>
     <mergeCell ref="D95:E95"/>
-    <mergeCell ref="C10:D10"/>
     <mergeCell ref="C76:E76"/>
     <mergeCell ref="A114:G114"/>
     <mergeCell ref="C93:G93"/>

</xml_diff>

<commit_message>
fix(contracts): restore browser print formatting
Apply template styles through CSSOM while preserving the inherited admin security policy. Remove seven trailing quotes from the client workbook and cover print styles and wording in focused tests.

Validation: 54 frontend tests, 3 renderer tests, scoped TypeScript checks, and Windows Edge PDF pagination with regular and long fields.
</commit_message>
<xml_diff>
--- a/db/templates/contracts/contract_client_copy.xlsx
+++ b/db/templates/contracts/contract_client_copy.xlsx
@@ -2117,7 +2117,7 @@
     <row r="13" ht="15" customHeight="1" s="148">
       <c r="A13" s="18" t="inlineStr">
         <is>
-          <t>提供合法合規之照顧服務媒合與管理。"</t>
+          <t>提供合法合規之照顧服務媒合與管理。</t>
         </is>
       </c>
       <c r="B13" s="150" t="n"/>
@@ -2130,7 +2130,7 @@
     <row r="14" ht="15" customHeight="1" s="148">
       <c r="A14" s="18" t="inlineStr">
         <is>
-          <t>建立服務品質監督機制，包括隨機抽查與定期評估。"</t>
+          <t>建立服務品質監督機制，包括隨機抽查與定期評估。</t>
         </is>
       </c>
       <c r="B14" s="150" t="n"/>
@@ -2143,7 +2143,7 @@
     <row r="15" ht="15" customHeight="1" s="148">
       <c r="A15" s="18" t="inlineStr">
         <is>
-          <t>妥善保存並保護委託人及受照顧者之個人資料。"</t>
+          <t>妥善保存並保護委託人及受照顧者之個人資料。</t>
         </is>
       </c>
       <c r="B15" s="150" t="n"/>
@@ -2156,7 +2156,7 @@
     <row r="16" ht="15" customHeight="1" s="148">
       <c r="A16" s="18" t="inlineStr">
         <is>
-          <t>服務期間提供服務人員意外責任險。"</t>
+          <t>服務期間提供服務人員意外責任險。</t>
         </is>
       </c>
       <c r="B16" s="150" t="n"/>
@@ -2182,7 +2182,7 @@
     <row r="18" ht="15" customHeight="1" s="148">
       <c r="A18" s="18" t="inlineStr">
         <is>
-          <t>得因委託人或受照顧者違反契約而終止服務。"</t>
+          <t>得因委託人或受照顧者違反契約而終止服務。</t>
         </is>
       </c>
       <c r="B18" s="150" t="n"/>
@@ -2195,7 +2195,7 @@
     <row r="19" ht="15" customHeight="1" s="148">
       <c r="A19" s="18" t="inlineStr">
         <is>
-          <t>得依政府規範調整服務內容與流程。"</t>
+          <t>得依政府規範調整服務內容與流程。</t>
         </is>
       </c>
       <c r="B19" s="150" t="n"/>
@@ -2221,7 +2221,7 @@
     <row r="21" ht="15" customHeight="1" s="148">
       <c r="A21" s="18" t="inlineStr">
         <is>
-          <t>委託人如未滿二十歲且未結婚，應得其法定代理人之同意，契約方生效。"</t>
+          <t>委託人如未滿二十歲且未結婚，應得其法定代理人之同意，契約方生效。</t>
         </is>
       </c>
       <c r="B21" s="150" t="n"/>

</xml_diff>